<commit_message>
feat: reasons.xlsx desteği, rapor ve scraper iyileştirmeleri, debug kodu kaldırıldı
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/urls.xlsx
+++ b/src/urls.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19580" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="URLs" sheetId="1" state="visible" r:id="rId1"/>
@@ -40,7 +40,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +97,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+        <bgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+        <bgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+        <bgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+        <bgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D6EAF8"/>
         <bgColor rgb="00D6EAF8"/>
       </patternFill>
@@ -108,7 +156,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -184,6 +232,79 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB0B0B0"/>
       </left>
@@ -195,13 +316,13 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
       <right style="thin">
         <color rgb="FFB0B0B0"/>
       </right>
-      <top style="thin">
-        <color rgb="FFB0B0B0"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color rgb="FFB0B0B0"/>
       </bottom>
@@ -223,32 +344,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB0B0B0"/>
-      </left>
+      <left/>
       <right style="thin">
         <color rgb="FFB0B0B0"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFB0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB0B0B0"/>
-      </left>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB0B0B0"/>
-      </right>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -305,7 +413,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -335,53 +443,141 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -748,7 +944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -816,7 +1012,7 @@
       </c>
     </row>
     <row r="2" ht="96" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
@@ -826,12 +1022,12 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="C2" s="43" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D2" s="43" t="inlineStr">
         <is>
           <t>5-5299000039410</t>
         </is>
@@ -864,10 +1060,10 @@
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="21" t="n"/>
+      <c r="A3" s="37" t="n"/>
       <c r="B3" s="10" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="17" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="29" t="n"/>
       <c r="E3" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/9zMQDXKJVzXpFw2A</t>
@@ -898,20 +1094,20 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/zR2BQ2sGghmETJTw9</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>Melodi Cafe Aliağa</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>9-0053000040115</t>
         </is>
@@ -946,10 +1142,10 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
+      <c r="A5" s="32" t="n"/>
+      <c r="B5" s="32" t="n"/>
+      <c r="C5" s="32" t="n"/>
+      <c r="D5" s="32" t="n"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/UQ9LxvTCZdLxumbz9</t>
@@ -980,10 +1176,10 @@
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
+      <c r="A6" s="32" t="n"/>
+      <c r="B6" s="32" t="n"/>
+      <c r="C6" s="32" t="n"/>
+      <c r="D6" s="32" t="n"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/hvhqBh7B1S1HANWg6</t>
@@ -1014,10 +1210,10 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="17" t="n"/>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
+      <c r="A7" s="29" t="n"/>
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/YaxU3dP4S3Yzx1gA6</t>
@@ -1048,20 +1244,20 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="45" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/qbE1nuEeBcSPYd7F8</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="B8" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
         <is>
           <t>Yeşil Döner Salonu</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="46" t="inlineStr">
         <is>
           <t>8-3100000039993</t>
         </is>
@@ -1096,10 +1292,10 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="17" t="n"/>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
+      <c r="A9" s="29" t="n"/>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/4U86oawUopyWAacM8</t>
@@ -1130,20 +1326,20 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C10" s="48" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="48" t="inlineStr">
         <is>
           <t>3-4885000039881</t>
         </is>
@@ -1178,10 +1374,10 @@
       </c>
     </row>
     <row r="11" ht="96" customHeight="1">
-      <c r="A11" s="17" t="n"/>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
+      <c r="A11" s="29" t="n"/>
+      <c r="B11" s="29" t="n"/>
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
       <c r="E11" s="13" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/zspqmDfq42ZboePX7</t>
@@ -1212,111 +1408,927 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D12" s="25" t="inlineStr">
+      <c r="D12" s="49" t="inlineStr">
         <is>
           <t>5-4398000039780</t>
         </is>
       </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/oberrv5dBj2Tb7h38</t>
         </is>
       </c>
-      <c r="F12" s="26" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>08.02.2026</t>
         </is>
       </c>
-      <c r="G12" s="26" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>Alp E. Bağcı</t>
         </is>
       </c>
-      <c r="H12" s="26" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Çikolata konusunda gayet başarılı olan bu markanın Etiler'deki kafesi. çayları ve tatlıları gayet lezzetli ve çalışanları güleryüzlü.</t>
         </is>
       </c>
-      <c r="I12" s="26" t="n">
+      <c r="I12" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="27" t="inlineStr">
-        <is>
-          <t>beklemede</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="28" t="n"/>
-      <c r="B13" s="28" t="n"/>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="64" customHeight="1">
+      <c r="A13" s="29" t="n"/>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/pRMboShfp197cc4t8</t>
         </is>
       </c>
-      <c r="F13" s="29" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>08.02.2026</t>
         </is>
       </c>
-      <c r="G13" s="29" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Gurme Rehber</t>
         </is>
       </c>
-      <c r="H13" s="29" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>Melodi Cafe, Etiler'de bulunan bir kafe. Burası Melodi Çikolata markasının açtığı ilk kafe ve son derece taze/lezzetli Melodi ürünlerini servis ediyorlar. Gittiğimizde hemen her ürünlerini deneme fırsatı yakaladık. Tatlı kurabiyeler, tuzlu …</t>
         </is>
       </c>
-      <c r="I13" s="29" t="n">
+      <c r="I13" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="J13" s="27" t="inlineStr">
-        <is>
-          <t>beklemede</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="E14" s="8" t="n"/>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="50" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
+        </is>
+      </c>
+      <c r="B14" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="51" t="inlineStr">
+        <is>
+          <t>Emre Etliekmek-Lahmacun / Meram</t>
+        </is>
+      </c>
+      <c r="D14" s="51" t="inlineStr">
+        <is>
+          <t>7-1001000040622</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/9fhnQpLVkADUMBJf8</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>Gurme Miki</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Bunlardan başka meze var mı dediğimde yok dediler, aynı menüyü söylediğimiz önümdeki masaya birkaç meze daha koydular, 2 tane turşu koysan ne eksilirsin, bu kadar fakirsen parasıyla ver ama varsa yok deme?yorumlar kendi çevresi olmalı ki …</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/H6Gn3ncRjT8DCu5u8</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>Ebru ÇAKIR</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
+        <is>
+          <t>Malesef adına emeğine güvenerek başka semtten gidip yaptırdığımız etliekmek .kalın bir hamur ,içi az ve yanık … bugün bu etliekmeği yapan ocak başındaki ustaya selam 👋🏻 bir müşteri kaybetmek sadece bi müşteri kaybetmek değildir aklınızda bulunsun …</t>
+        </is>
+      </c>
+      <c r="I15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="32" t="n"/>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/YQtrUjEWjAuFKTLK8</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>Wrd</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Nakit veya ibandan ödeme almak için pos cihazında sürekli problem olan işletme. Son gidişimiz oldu.</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="32" t="n"/>
+      <c r="B17" s="32" t="n"/>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="32" t="n"/>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/6TbjSJE5FVbf79MW8</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>Rüveyda Erdoğan</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>Burada ıspanaklı börek yaptırdık ve üzerine yumurta kırmalarını istedik. Ancak, yumurtaları kabuklarıyla birlikte iç harcına koymuşlar! Eve geldiğimizde böreklerin içinde yumurta kabukları vardı. Hatalarını telafi etmeleri için geri …</t>
+        </is>
+      </c>
+      <c r="I17" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="64" customHeight="1">
+      <c r="A18" s="32" t="n"/>
+      <c r="B18" s="32" t="n"/>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/xsUGvK1mWCuLxSwo6</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Sait Eroglu</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Meram itfaiye yanındaki şubesinin yaptığı etli ekmek  bu nimete sözüm yok ama yapan tam bir odunmus birdaha asla işim olmaz aklı olan gitmez. Istanbuldan geldim etli ekmek yeriz diye lahmacunu mumla aradik</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="64" customHeight="1">
+      <c r="A19" s="32" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/6nm5nuKveuj4WGUg7</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>Ahmet</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>Arkadaşlarımın tavsiyesi üzerine gittik lahmacun güzel fakat servis anlamında çok kötü, 4 lahmacun tam 30 dakikada geldi, dolaplarında litrelik ayran var müşteriye veremeyiz diyorlar ben böyle bir işletme görmedim</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="32" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/DEZhm5ty9VieEaqA8</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>RN MR</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Bi iftar yapalım dedik tesadüf girdik 2 az çorba 2 adet 1 er buçuk etli ekmek 1ltre ayran 300₺ tuttu. Bayağı bayağı abartı bi fiyat. Ekli ekmek tatsız tuzsuz içi bol ama lezzet yok.</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="32" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/H9BTnikxNQFtWtra7</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G21" s="21" t="inlineStr">
+        <is>
+          <t>Mustafa Küçükbezirci</t>
+        </is>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Berbat biryer asla tavsiye etmiyorum ne yemekleri ne esnaflık asla ve alsa gidilmemesi gereken bir yer</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="64" customHeight="1">
+      <c r="A22" s="32" t="n"/>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/zbwwzY43og7Dh9yA9</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Fadimana Gençarslan</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Gerçekten iğrençsiniz. Siparişi vereli 2 saat oldu ne yemek var ne de özür.  Bir de teslim edildi gösteriyorlar. Işinizi hakkıyla yapmanızı öneririm.  Zira haram lokma. Belki siz yemeye alışkınsınızdır ama mübarek günlerde yapmayın bari</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="29" t="n"/>
+      <c r="B23" s="29" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/Mi8ZcXBq1v7P9qpE8</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G23" s="21" t="inlineStr">
+        <is>
+          <t>uğur can yıldız</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>Dışarıdan paket siparişi geldiğinde sizin yaptırdığınız etliekmek arka sıraya alınıyor. Böylece geç yapılıyor.</t>
+        </is>
+      </c>
+      <c r="I23" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="20" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="53" t="inlineStr">
+        <is>
+          <t>Emre Etliekmek-Lahmacun / Meram</t>
+        </is>
+      </c>
+      <c r="D24" s="53" t="inlineStr">
+        <is>
+          <t>2-7618000039663</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/kDtW2FapwAKp5xP59</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>Osman Bolcan</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>Bir kere etli ekmek yaptırmıştım ve beğenmemiştim ama asıl bomba yağ somunu. Bu yediğim yağ somunu değil bildiğiniz en kötü tost veya ekmek arası ısıtılmış kaşar. Elinize sağlık diyemeyeceğim kusura bakmayın. Daha da gitmem</t>
+        </is>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="23" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="32" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/z5uaVHLRyXEJnZYH6</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>Mateja Ali</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
+        <is>
+          <t>İçerde yersen hamur var iç getirirsen hamur yok! Konya'da bu adet yeni çıktı herhalde?</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="23" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="64" customHeight="1">
+      <c r="A26" s="32" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/jSRUEGw9mWmPqyJt9</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>Hilal Yılmaz</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>6 yaş oğlumu ve 60 yaş şekeri düşmüş annemi akşam saatlerinde çok acıktıkları için etliekmek yemeye götürdüm. Elemanları önümüze üstte birkaç iyi ama alttakileri yanmış kömür olmuş kara pideler getirdi. …</t>
+        </is>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="23" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="32" t="n"/>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/z1ag5e3C7ZhNE2iZ6</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>Murat Mert Yıldız</t>
+        </is>
+      </c>
+      <c r="H27" s="24" t="inlineStr">
+        <is>
+          <t>Çok kötü Bi yer çok pis sipariş veriyoruz gelmiyor sürekli çıkıyor çıkıyor diye oyalıyorlar</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="23" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="64" customHeight="1">
+      <c r="A28" s="29" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/ogA8r6KRPnHv1PPR8</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>Ayşe Kara</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Hiç beğenmedim bidaha kesinlikle gitmem. Çok bekletiliyorum çalışanlar yavaş çalışılıyorlar ve telefon oynuyorlar sürekli, müşteriyle ilgilenmiyorlar.
+Yani kısacası kesinlikle gitmeyin derim.</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="23" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="80" customHeight="1">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Emre Etliekmek-Lahmacun / Meram</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>2-5803000040380</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/pWNrLbJabZ41yYrX9</t>
+        </is>
+      </c>
+      <c r="F29" s="25" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>Ebru ÇAKIR</t>
+        </is>
+      </c>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>Malesef adına emeğine güvenerek başka semtten gidip yaptırdığımız etliekmek .kalın bir hamur ,içi az ve yanık … bugün bu etliekmeği yapan ocak başındaki ustaya selam 👋🏻 bir müşteri kaybetmek sadece bi müşteri kaybetmek değildir aklınızda bulunsun …</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>Emre Etliekmek-Lahmacun / Meram</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>2-5803000040380</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/Vi57QoVCQ7WXg8MK7</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>Wrd</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="inlineStr">
+        <is>
+          <t>Nakit veya ibandan ödeme almak için pos cihazında sürekli problem olan işletme. Son gidişimiz oldu.</t>
+        </is>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="26" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="64" customHeight="1">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>Emre Etliekmek-Lahmacun / Meram</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>2-5803000040380</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/RgqYnVuU3cNbPJAbA</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>Rüveyda Erdoğan</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>Burada ıspanaklı börek yaptırdık ve üzerine yumurta kırmalarını istedik. Ancak, yumurtaları kabuklarıyla birlikte iç harcına koymuşlar! Eve geldiğimizde böreklerin içinde yumurta kabukları vardı. Hatalarını telafi etmeleri için geri …</t>
+        </is>
+      </c>
+      <c r="I31" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="26" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="54" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/Z6cbgLJDuJ7RCgUb6</t>
+        </is>
+      </c>
+      <c r="B32" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="55" t="inlineStr">
+        <is>
+          <t>Koff Coffee Company</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="inlineStr">
+        <is>
+          <t>5-6135000040494</t>
+        </is>
+      </c>
+      <c r="E32" s="55" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/7EPznGLd4mkwVgUx8</t>
+        </is>
+      </c>
+      <c r="F32" s="55" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G32" s="55" t="inlineStr">
+        <is>
+          <t>sena tuğlu</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>eskiden arkadaşlarımla buluşmak ve çalışmak için sık tercih ettiğim bir yerdi. kahve/tatlı/ortam olarak f/p buluyordum. 1 ay önce arkadaşımla tercih ettiğimizde hem tatlı çeşidi yoktu hem internetlerinde problem vardı. bugün kahve alırken …</t>
+        </is>
+      </c>
+      <c r="I32" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="56" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="57" t="n"/>
+      <c r="B33" s="57" t="n"/>
+      <c r="C33" s="58" t="inlineStr">
+        <is>
+          <t>Koff Coffee Company</t>
+        </is>
+      </c>
+      <c r="D33" s="57" t="n"/>
+      <c r="E33" s="58" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/cCavG7dj7w9a9qy57</t>
+        </is>
+      </c>
+      <c r="F33" s="58" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G33" s="58" t="inlineStr">
+        <is>
+          <t>Eren Unuvar</t>
+        </is>
+      </c>
+      <c r="H33" s="58" t="inlineStr">
+        <is>
+          <t>Soğuk filtre kahvesi bayat muhtemelen 1 haftalık demleyip dolaba atıyorlar içine de buzu basıp satıyorlar.
+Keşke bayat olduğunu söyleselerdi.</t>
+        </is>
+      </c>
+      <c r="I33" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="56" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="59" t="n"/>
+      <c r="B34" s="59" t="n"/>
+      <c r="C34" s="55" t="inlineStr">
+        <is>
+          <t>Koff Coffee Company</t>
+        </is>
+      </c>
+      <c r="D34" s="59" t="n"/>
+      <c r="E34" s="55" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/VCGgJyKNoh6xQgN38</t>
+        </is>
+      </c>
+      <c r="F34" s="55" t="inlineStr">
+        <is>
+          <t>27.02.2026</t>
+        </is>
+      </c>
+      <c r="G34" s="55" t="inlineStr">
+        <is>
+          <t>fatih</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>arkadaşımla hibiscus ve fresh lime almıştık ama tadları içilmiycek kadar kötü dimesin cool limei ile yapsalar bin kat daha güzel olurdu hibiscusda sadece şeker ve su tadı geliyor ve ice americano ile değiştirmelerini istedik lakin yüzüme …</t>
+        </is>
+      </c>
+      <c r="I34" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="56" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="30">
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="B8:B9"/>
+    <mergeCell ref="D14:D23"/>
+    <mergeCell ref="A32:A34"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="C4:C7"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="C12:C13"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="D24:D28"/>
+    <mergeCell ref="C14:C23"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B32:B34"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="C24:C28"/>
     <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B14:B23"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A23"/>
+    <mergeCell ref="D32:D34"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Geçersiz Değer" error="Lütfen listeden bir değer seçin" promptTitle="Durum" prompt="Durum seçin" type="list">
@@ -1333,6 +2345,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: resimli yorumları otomatik atlama özelliği
Raporlanacak yorumlarda fotoğraf/resim tespit edilirse o yorum atlanıp
bir sonraki en kötü yoruma geçiliyor. Tekrar raporlamada da aynı mantık
çalışıyor.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/urls.xlsx
+++ b/src/urls.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2980" yWindow="1100" windowWidth="38400" windowHeight="19400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="URLs" sheetId="1" state="visible" r:id="rId1"/>
@@ -40,7 +40,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -145,18 +145,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
-        <bgColor rgb="00D6EAF8"/>
+        <fgColor rgb="FFD6EAF8"/>
+        <bgColor rgb="FFD6EAF8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -344,7 +350,24 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
       <right style="thin">
         <color rgb="FFB0B0B0"/>
       </right>
@@ -356,28 +379,18 @@
       <left style="thin">
         <color rgb="FFB0B0B0"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </left>
       <right/>
       <top/>
@@ -385,27 +398,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -413,7 +411,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -494,90 +492,93 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -944,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1012,7 +1013,7 @@
       </c>
     </row>
     <row r="2" ht="96" customHeight="1">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
@@ -1022,12 +1023,12 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C2" s="43" t="inlineStr">
+      <c r="C2" s="49" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D2" s="43" t="inlineStr">
+      <c r="D2" s="49" t="inlineStr">
         <is>
           <t>5-5299000039410</t>
         </is>
@@ -1060,10 +1061,10 @@
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="37" t="n"/>
+      <c r="A3" s="43" t="n"/>
       <c r="B3" s="10" t="n"/>
-      <c r="C3" s="29" t="n"/>
-      <c r="D3" s="29" t="n"/>
+      <c r="C3" s="38" t="n"/>
+      <c r="D3" s="38" t="n"/>
       <c r="E3" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/9zMQDXKJVzXpFw2A</t>
@@ -1094,20 +1095,20 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/zR2BQ2sGghmETJTw9</t>
         </is>
       </c>
-      <c r="B4" s="43" t="n">
+      <c r="B4" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="43" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Melodi Cafe Aliağa</t>
         </is>
       </c>
-      <c r="D4" s="43" t="inlineStr">
+      <c r="D4" s="49" t="inlineStr">
         <is>
           <t>9-0053000040115</t>
         </is>
@@ -1142,10 +1143,10 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="32" t="n"/>
-      <c r="B5" s="32" t="n"/>
-      <c r="C5" s="32" t="n"/>
-      <c r="D5" s="32" t="n"/>
+      <c r="A5" s="37" t="n"/>
+      <c r="B5" s="37" t="n"/>
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="37" t="n"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/UQ9LxvTCZdLxumbz9</t>
@@ -1176,10 +1177,10 @@
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="32" t="n"/>
-      <c r="B6" s="32" t="n"/>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="32" t="n"/>
+      <c r="A6" s="37" t="n"/>
+      <c r="B6" s="37" t="n"/>
+      <c r="C6" s="37" t="n"/>
+      <c r="D6" s="37" t="n"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/hvhqBh7B1S1HANWg6</t>
@@ -1210,10 +1211,10 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="29" t="n"/>
-      <c r="B7" s="29" t="n"/>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="29" t="n"/>
+      <c r="A7" s="38" t="n"/>
+      <c r="B7" s="38" t="n"/>
+      <c r="C7" s="38" t="n"/>
+      <c r="D7" s="38" t="n"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/YaxU3dP4S3Yzx1gA6</t>
@@ -1244,20 +1245,20 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="45" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/qbE1nuEeBcSPYd7F8</t>
         </is>
       </c>
-      <c r="B8" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="46" t="inlineStr">
+      <c r="B8" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="52" t="inlineStr">
         <is>
           <t>Yeşil Döner Salonu</t>
         </is>
       </c>
-      <c r="D8" s="46" t="inlineStr">
+      <c r="D8" s="52" t="inlineStr">
         <is>
           <t>8-3100000039993</t>
         </is>
@@ -1292,10 +1293,10 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
+      <c r="A9" s="38" t="n"/>
+      <c r="B9" s="38" t="n"/>
+      <c r="C9" s="38" t="n"/>
+      <c r="D9" s="38" t="n"/>
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/4U86oawUopyWAacM8</t>
@@ -1326,20 +1327,20 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="47" t="inlineStr">
+      <c r="A10" s="53" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
       </c>
-      <c r="B10" s="48" t="n">
+      <c r="B10" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D10" s="48" t="inlineStr">
+      <c r="D10" s="54" t="inlineStr">
         <is>
           <t>3-4885000039881</t>
         </is>
@@ -1374,10 +1375,10 @@
       </c>
     </row>
     <row r="11" ht="96" customHeight="1">
-      <c r="A11" s="29" t="n"/>
-      <c r="B11" s="29" t="n"/>
-      <c r="C11" s="29" t="n"/>
-      <c r="D11" s="29" t="n"/>
+      <c r="A11" s="38" t="n"/>
+      <c r="B11" s="38" t="n"/>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="38" t="n"/>
       <c r="E11" s="13" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/zspqmDfq42ZboePX7</t>
@@ -1408,20 +1409,20 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="55" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/X9r6LfdgGrrYWRKz9</t>
         </is>
       </c>
-      <c r="B12" s="49" t="n">
+      <c r="B12" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="49" t="inlineStr">
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>Melodi Cafe</t>
         </is>
       </c>
-      <c r="D12" s="49" t="inlineStr">
+      <c r="D12" s="55" t="inlineStr">
         <is>
           <t>5-4398000039780</t>
         </is>
@@ -1456,10 +1457,10 @@
       </c>
     </row>
     <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="29" t="n"/>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
+      <c r="A13" s="38" t="n"/>
+      <c r="B13" s="38" t="n"/>
+      <c r="C13" s="38" t="n"/>
+      <c r="D13" s="38" t="n"/>
       <c r="E13" s="17" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/pRMboShfp197cc4t8</t>
@@ -1490,20 +1491,20 @@
       </c>
     </row>
     <row r="14" ht="80" customHeight="1">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
         </is>
       </c>
-      <c r="B14" s="51" t="n">
+      <c r="B14" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="C14" s="51" t="inlineStr">
+      <c r="C14" s="57" t="inlineStr">
         <is>
           <t>Emre Etliekmek-Lahmacun / Meram</t>
         </is>
       </c>
-      <c r="D14" s="51" t="inlineStr">
+      <c r="D14" s="57" t="inlineStr">
         <is>
           <t>7-1001000040622</t>
         </is>
@@ -1538,10 +1539,10 @@
       </c>
     </row>
     <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="32" t="n"/>
-      <c r="B15" s="32" t="n"/>
-      <c r="C15" s="32" t="n"/>
-      <c r="D15" s="32" t="n"/>
+      <c r="A15" s="37" t="n"/>
+      <c r="B15" s="37" t="n"/>
+      <c r="C15" s="37" t="n"/>
+      <c r="D15" s="37" t="n"/>
       <c r="E15" s="21" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/H6Gn3ncRjT8DCu5u8</t>
@@ -1572,10 +1573,10 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="32" t="n"/>
-      <c r="B16" s="32" t="n"/>
-      <c r="C16" s="32" t="n"/>
-      <c r="D16" s="32" t="n"/>
+      <c r="A16" s="37" t="n"/>
+      <c r="B16" s="37" t="n"/>
+      <c r="C16" s="37" t="n"/>
+      <c r="D16" s="37" t="n"/>
       <c r="E16" s="19" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/YQtrUjEWjAuFKTLK8</t>
@@ -1599,17 +1600,17 @@
       <c r="I16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="20" t="inlineStr">
-        <is>
-          <t>beklemede</t>
+      <c r="J16" s="58" t="inlineStr">
+        <is>
+          <t>silindi</t>
         </is>
       </c>
     </row>
     <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="32" t="n"/>
-      <c r="B17" s="32" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
+      <c r="A17" s="37" t="n"/>
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="37" t="n"/>
+      <c r="D17" s="37" t="n"/>
       <c r="E17" s="21" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/6TbjSJE5FVbf79MW8</t>
@@ -1640,10 +1641,10 @@
       </c>
     </row>
     <row r="18" ht="64" customHeight="1">
-      <c r="A18" s="32" t="n"/>
-      <c r="B18" s="32" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
+      <c r="A18" s="37" t="n"/>
+      <c r="B18" s="37" t="n"/>
+      <c r="C18" s="37" t="n"/>
+      <c r="D18" s="37" t="n"/>
       <c r="E18" s="19" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/xsUGvK1mWCuLxSwo6</t>
@@ -1674,10 +1675,10 @@
       </c>
     </row>
     <row r="19" ht="64" customHeight="1">
-      <c r="A19" s="32" t="n"/>
-      <c r="B19" s="32" t="n"/>
-      <c r="C19" s="32" t="n"/>
-      <c r="D19" s="32" t="n"/>
+      <c r="A19" s="37" t="n"/>
+      <c r="B19" s="37" t="n"/>
+      <c r="C19" s="37" t="n"/>
+      <c r="D19" s="37" t="n"/>
       <c r="E19" s="21" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/6nm5nuKveuj4WGUg7</t>
@@ -1708,10 +1709,10 @@
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="32" t="n"/>
-      <c r="B20" s="32" t="n"/>
-      <c r="C20" s="32" t="n"/>
-      <c r="D20" s="32" t="n"/>
+      <c r="A20" s="37" t="n"/>
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="37" t="n"/>
+      <c r="D20" s="37" t="n"/>
       <c r="E20" s="19" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/DEZhm5ty9VieEaqA8</t>
@@ -1742,10 +1743,10 @@
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="32" t="n"/>
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
+      <c r="A21" s="37" t="n"/>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="37" t="n"/>
+      <c r="D21" s="37" t="n"/>
       <c r="E21" s="21" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/H9BTnikxNQFtWtra7</t>
@@ -1776,10 +1777,10 @@
       </c>
     </row>
     <row r="22" ht="64" customHeight="1">
-      <c r="A22" s="32" t="n"/>
-      <c r="B22" s="32" t="n"/>
-      <c r="C22" s="32" t="n"/>
-      <c r="D22" s="32" t="n"/>
+      <c r="A22" s="37" t="n"/>
+      <c r="B22" s="37" t="n"/>
+      <c r="C22" s="37" t="n"/>
+      <c r="D22" s="37" t="n"/>
       <c r="E22" s="19" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/zbwwzY43og7Dh9yA9</t>
@@ -1810,10 +1811,10 @@
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="29" t="n"/>
-      <c r="B23" s="29" t="n"/>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="29" t="n"/>
+      <c r="A23" s="38" t="n"/>
+      <c r="B23" s="38" t="n"/>
+      <c r="C23" s="38" t="n"/>
+      <c r="D23" s="38" t="n"/>
       <c r="E23" s="21" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/Mi8ZcXBq1v7P9qpE8</t>
@@ -1844,20 +1845,20 @@
       </c>
     </row>
     <row r="24" ht="64" customHeight="1">
-      <c r="A24" s="52" t="inlineStr">
+      <c r="A24" s="59" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/g6VDRuWyAE51HJGf6</t>
         </is>
       </c>
-      <c r="B24" s="53" t="n">
+      <c r="B24" s="60" t="n">
         <v>5</v>
       </c>
-      <c r="C24" s="53" t="inlineStr">
+      <c r="C24" s="60" t="inlineStr">
         <is>
           <t>Emre Etliekmek-Lahmacun / Meram</t>
         </is>
       </c>
-      <c r="D24" s="53" t="inlineStr">
+      <c r="D24" s="60" t="inlineStr">
         <is>
           <t>2-7618000039663</t>
         </is>
@@ -1892,10 +1893,10 @@
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="32" t="n"/>
-      <c r="B25" s="32" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
+      <c r="A25" s="37" t="n"/>
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="37" t="n"/>
+      <c r="D25" s="37" t="n"/>
       <c r="E25" s="24" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/z5uaVHLRyXEJnZYH6</t>
@@ -1926,10 +1927,10 @@
       </c>
     </row>
     <row r="26" ht="64" customHeight="1">
-      <c r="A26" s="32" t="n"/>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
+      <c r="A26" s="37" t="n"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="37" t="n"/>
+      <c r="D26" s="37" t="n"/>
       <c r="E26" s="22" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/jSRUEGw9mWmPqyJt9</t>
@@ -1960,10 +1961,10 @@
       </c>
     </row>
     <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="32" t="n"/>
-      <c r="B27" s="32" t="n"/>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="32" t="n"/>
+      <c r="A27" s="37" t="n"/>
+      <c r="B27" s="37" t="n"/>
+      <c r="C27" s="37" t="n"/>
+      <c r="D27" s="37" t="n"/>
       <c r="E27" s="24" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/z1ag5e3C7ZhNE2iZ6</t>
@@ -1994,10 +1995,10 @@
       </c>
     </row>
     <row r="28" ht="64" customHeight="1">
-      <c r="A28" s="29" t="n"/>
-      <c r="B28" s="29" t="n"/>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="29" t="n"/>
+      <c r="A28" s="38" t="n"/>
+      <c r="B28" s="38" t="n"/>
+      <c r="C28" s="38" t="n"/>
+      <c r="D28" s="38" t="n"/>
       <c r="E28" s="22" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/ogA8r6KRPnHv1PPR8</t>
@@ -2172,129 +2173,139 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="54" t="inlineStr">
+    <row r="32" ht="64" customHeight="1">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/Z6cbgLJDuJ7RCgUb6</t>
         </is>
       </c>
-      <c r="B32" s="54" t="n">
+      <c r="B32" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="C32" s="55" t="inlineStr">
+      <c r="C32" s="28" t="inlineStr">
         <is>
           <t>Koff Coffee Company</t>
         </is>
       </c>
-      <c r="D32" s="54" t="inlineStr">
+      <c r="D32" s="36" t="inlineStr">
         <is>
           <t>5-6135000040494</t>
         </is>
       </c>
-      <c r="E32" s="55" t="inlineStr">
+      <c r="E32" s="28" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/7EPznGLd4mkwVgUx8</t>
         </is>
       </c>
-      <c r="F32" s="55" t="inlineStr">
+      <c r="F32" s="28" t="inlineStr">
         <is>
           <t>27.02.2026</t>
         </is>
       </c>
-      <c r="G32" s="55" t="inlineStr">
+      <c r="G32" s="28" t="inlineStr">
         <is>
           <t>sena tuğlu</t>
         </is>
       </c>
-      <c r="H32" s="55" t="inlineStr">
+      <c r="H32" s="28" t="inlineStr">
         <is>
           <t>eskiden arkadaşlarımla buluşmak ve çalışmak için sık tercih ettiğim bir yerdi. kahve/tatlı/ortam olarak f/p buluyordum. 1 ay önce arkadaşımla tercih ettiğimizde hem tatlı çeşidi yoktu hem internetlerinde problem vardı. bugün kahve alırken …</t>
         </is>
       </c>
-      <c r="I32" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="56" t="inlineStr">
-        <is>
-          <t>beklemede</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="57" t="n"/>
-      <c r="B33" s="57" t="n"/>
-      <c r="C33" s="58" t="inlineStr">
+      <c r="I32" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="29" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="37" t="n"/>
+      <c r="B33" s="37" t="n"/>
+      <c r="C33" s="30" t="inlineStr">
         <is>
           <t>Koff Coffee Company</t>
         </is>
       </c>
-      <c r="D33" s="57" t="n"/>
-      <c r="E33" s="58" t="inlineStr">
+      <c r="D33" s="37" t="n"/>
+      <c r="E33" s="30" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/cCavG7dj7w9a9qy57</t>
         </is>
       </c>
-      <c r="F33" s="58" t="inlineStr">
+      <c r="F33" s="30" t="inlineStr">
         <is>
           <t>27.02.2026</t>
         </is>
       </c>
-      <c r="G33" s="58" t="inlineStr">
+      <c r="G33" s="30" t="inlineStr">
         <is>
           <t>Eren Unuvar</t>
         </is>
       </c>
-      <c r="H33" s="58" t="inlineStr">
+      <c r="H33" s="30" t="inlineStr">
         <is>
           <t>Soğuk filtre kahvesi bayat muhtemelen 1 haftalık demleyip dolaba atıyorlar içine de buzu basıp satıyorlar.
 Keşke bayat olduğunu söyleselerdi.</t>
         </is>
       </c>
-      <c r="I33" s="58" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="56" t="inlineStr">
-        <is>
-          <t>beklemede</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="59" t="n"/>
-      <c r="B34" s="59" t="n"/>
-      <c r="C34" s="55" t="inlineStr">
+      <c r="I33" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="29" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="64" customHeight="1">
+      <c r="A34" s="38" t="n"/>
+      <c r="B34" s="38" t="n"/>
+      <c r="C34" s="28" t="inlineStr">
         <is>
           <t>Koff Coffee Company</t>
         </is>
       </c>
-      <c r="D34" s="59" t="n"/>
-      <c r="E34" s="55" t="inlineStr">
+      <c r="D34" s="38" t="n"/>
+      <c r="E34" s="28" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/VCGgJyKNoh6xQgN38</t>
         </is>
       </c>
-      <c r="F34" s="55" t="inlineStr">
+      <c r="F34" s="28" t="inlineStr">
         <is>
           <t>27.02.2026</t>
         </is>
       </c>
-      <c r="G34" s="55" t="inlineStr">
+      <c r="G34" s="28" t="inlineStr">
         <is>
           <t>fatih</t>
         </is>
       </c>
-      <c r="H34" s="55" t="inlineStr">
+      <c r="H34" s="28" t="inlineStr">
         <is>
           <t>arkadaşımla hibiscus ve fresh lime almıştık ama tadları içilmiycek kadar kötü dimesin cool limei ile yapsalar bin kat daha güzel olurdu hibiscusda sadece şeker ve su tadı geliyor ve ice americano ile değiştirmelerini istedik lakin yüzüme …</t>
         </is>
       </c>
-      <c r="I34" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" s="56" t="inlineStr">
-        <is>
-          <t>beklemede</t>
-        </is>
+      <c r="I34" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="29" t="inlineStr">
+        <is>
+          <t>beklemede</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/o4QEuxrh39JXskhn7</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: humanize toggle, JWT token doğrulama, EXE build iyileştirmesi
- Human-like browser davranışları artık --humanize flag'i ile toggle edilebilir (varsayılan: kapalı)
- Rapor gönderimi sonrası Lambda validate-token endpoint'ine JWT ile doğrulama eklendi
- PyJWT hidden import EXE build workflow'una eklendi

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/urls.xlsx
+++ b/src/urls.xlsx
@@ -411,7 +411,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -578,6 +578,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2023,9 +2032,9 @@
       <c r="I28" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="23" t="inlineStr">
-        <is>
-          <t>beklemede</t>
+      <c r="J28" s="61" t="inlineStr">
+        <is>
+          <t>silindi</t>
         </is>
       </c>
     </row>
@@ -2119,9 +2128,9 @@
       <c r="I30" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="J30" s="26" t="inlineStr">
-        <is>
-          <t>beklemede</t>
+      <c r="J30" s="62" t="inlineStr">
+        <is>
+          <t>silindi</t>
         </is>
       </c>
     </row>
@@ -2254,9 +2263,9 @@
       <c r="I33" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="29" t="inlineStr">
-        <is>
-          <t>beklemede</t>
+      <c r="J33" s="63" t="inlineStr">
+        <is>
+          <t>silindi</t>
         </is>
       </c>
     </row>

</xml_diff>